<commit_message>
Illustrative README: restore sections required by tests (top customers, open invoices, planned payments, recurring outflows); demo data rebuilt from latest engine outputs (S7 actuals pending re-export)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXUr26jGf9sv6ye7xasg2x
</commit_message>
<xml_diff>
--- a/frontend/demo/sample/S7_sample_dataset.xlsx
+++ b/frontend/demo/sample/S7_sample_dataset.xlsx
@@ -749,10 +749,10 @@
         <v>1200000</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>663883</v>
+        <v>655195</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>126692</v>
+        <v>23413</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>0</v>
@@ -767,25 +767,25 @@
         <v>0</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>451692</v>
+        <v>348413</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>1412191</v>
+        <v>1506782</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>1233531</v>
+        <v>1331737</v>
       </c>
       <c r="M5" s="11" t="n">
-        <v>1583723</v>
+        <v>1693669</v>
       </c>
       <c r="N5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="11" t="n">
-        <v>1813769</v>
+        <v>1904398</v>
       </c>
       <c r="P5" s="11" t="n">
-        <v>1240093</v>
+        <v>1346443</v>
       </c>
       <c r="Q5" s="11" t="n">
         <v>509538</v>
@@ -802,13 +802,13 @@
         <v>46300</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1412191</v>
+        <v>1506782</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>502383</v>
+        <v>509437</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>76457</v>
+        <v>348556</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
@@ -823,25 +823,25 @@
         <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>126457</v>
+        <v>398556</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>1788116</v>
+        <v>1617663</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>1584245</v>
+        <v>1427387</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>1982484</v>
+        <v>1825841</v>
       </c>
       <c r="N6" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2491956</v>
+        <v>2320993</v>
       </c>
       <c r="P6" s="11" t="n">
-        <v>1615961</v>
+        <v>1455194</v>
       </c>
       <c r="Q6" s="11" t="n">
         <v>509538</v>
@@ -858,13 +858,13 @@
         <v>46307</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1788116</v>
+        <v>1617663</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>519418</v>
+        <v>526208</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>1135714</v>
+        <v>696024</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0</v>
@@ -876,28 +876,28 @@
         <v>177000</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>105988</v>
+        <v>80341</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>1418702</v>
+        <v>953365</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>888832</v>
+        <v>1190506</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>688405</v>
+        <v>985487</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>1080238</v>
+        <v>1377785</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>0.013</v>
+        <v>0</v>
       </c>
       <c r="O7" s="11" t="n">
-        <v>1767374</v>
+        <v>2063185</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>717178</v>
+        <v>1020976</v>
       </c>
       <c r="Q7" s="11" t="n">
         <v>509538</v>
@@ -914,13 +914,13 @@
         <v>46314</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>888832</v>
+        <v>1190506</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>517190</v>
+        <v>514543</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>339048</v>
+        <v>400886</v>
       </c>
       <c r="F8" s="11" t="n">
         <v>0</v>
@@ -935,25 +935,25 @@
         <v>0</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>339048</v>
+        <v>400886</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>1066974</v>
+        <v>1304163</v>
       </c>
       <c r="L8" s="11" t="n">
-        <v>869828</v>
+        <v>1088251</v>
       </c>
       <c r="M8" s="11" t="n">
-        <v>1259616</v>
+        <v>1496896</v>
       </c>
       <c r="N8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="11" t="n">
-        <v>2079298</v>
+        <v>2314374</v>
       </c>
       <c r="P8" s="11" t="n">
-        <v>875400</v>
+        <v>1111897</v>
       </c>
       <c r="Q8" s="11" t="n">
         <v>509538</v>
@@ -970,13 +970,13 @@
         <v>46321</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1066974</v>
+        <v>1304163</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>568725</v>
+        <v>562359</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>26292</v>
+        <v>220496</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>81240</v>
@@ -991,25 +991,25 @@
         <v>0</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>432531</v>
+        <v>626736</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1203168</v>
+        <v>1239786</v>
       </c>
       <c r="L9" s="11" t="n">
-        <v>988287</v>
+        <v>1031582</v>
       </c>
       <c r="M9" s="11" t="n">
-        <v>1377163</v>
+        <v>1429094</v>
       </c>
       <c r="N9" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>2324189</v>
+        <v>2365998</v>
       </c>
       <c r="P9" s="11" t="n">
-        <v>979622</v>
+        <v>1034935</v>
       </c>
       <c r="Q9" s="11" t="n">
         <v>509538</v>
@@ -1026,10 +1026,10 @@
         <v>46328</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>1203168</v>
+        <v>1239786</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>485478</v>
+        <v>489009</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>0</v>
@@ -1050,22 +1050,22 @@
         <v>160521</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>1528125</v>
+        <v>1568274</v>
       </c>
       <c r="L10" s="11" t="n">
-        <v>1317560</v>
+        <v>1368398</v>
       </c>
       <c r="M10" s="11" t="n">
-        <v>1716465</v>
+        <v>1753770</v>
       </c>
       <c r="N10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2629126</v>
+        <v>2668964</v>
       </c>
       <c r="P10" s="11" t="n">
-        <v>1331895</v>
+        <v>1384948</v>
       </c>
       <c r="Q10" s="11" t="n">
         <v>509538</v>
@@ -1082,13 +1082,13 @@
         <v>46335</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>1528125</v>
+        <v>1568274</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>526404</v>
+        <v>523814</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>609811</v>
+        <v>799490</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>212459</v>
@@ -1103,25 +1103,25 @@
         <v>96457</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>1095726</v>
+        <v>1285406</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>958802</v>
+        <v>806683</v>
       </c>
       <c r="L11" s="11" t="n">
-        <v>751217</v>
+        <v>618727</v>
       </c>
       <c r="M11" s="11" t="n">
-        <v>1125202</v>
+        <v>981051</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>0.001</v>
+        <v>0.025</v>
       </c>
       <c r="O11" s="11" t="n">
-        <v>1979357</v>
+        <v>1831033</v>
       </c>
       <c r="P11" s="11" t="n">
-        <v>789747</v>
+        <v>655863</v>
       </c>
       <c r="Q11" s="11" t="n">
         <v>509538</v>
@@ -1138,10 +1138,10 @@
         <v>46342</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>958802</v>
+        <v>806683</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>474845</v>
+        <v>483045</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
@@ -1162,22 +1162,22 @@
         <v>247503</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>1186144</v>
+        <v>1042225</v>
       </c>
       <c r="L12" s="11" t="n">
-        <v>1003141</v>
+        <v>864854</v>
       </c>
       <c r="M12" s="11" t="n">
-        <v>1354325</v>
+        <v>1206929</v>
       </c>
       <c r="N12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="11" t="n">
-        <v>2039429</v>
+        <v>1889244</v>
       </c>
       <c r="P12" s="11" t="n">
-        <v>1054768</v>
+        <v>920043</v>
       </c>
       <c r="Q12" s="11" t="n">
         <v>509538</v>
@@ -1194,10 +1194,10 @@
         <v>46349</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>1186144</v>
+        <v>1042225</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>570564</v>
+        <v>568724</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>0</v>
@@ -1218,22 +1218,22 @@
         <v>350004</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>1406704</v>
+        <v>1260945</v>
       </c>
       <c r="L13" s="11" t="n">
-        <v>1238734</v>
+        <v>1102458</v>
       </c>
       <c r="M13" s="11" t="n">
-        <v>1551038</v>
+        <v>1399641</v>
       </c>
       <c r="N13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2059059</v>
+        <v>1911880</v>
       </c>
       <c r="P13" s="11" t="n">
-        <v>1327169</v>
+        <v>1199287</v>
       </c>
       <c r="Q13" s="11" t="n">
         <v>509538</v>
@@ -1250,10 +1250,10 @@
         <v>46356</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>1406704</v>
+        <v>1260945</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>666734</v>
+        <v>674838</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>0</v>
@@ -1274,22 +1274,22 @@
         <v>762112</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>1311325</v>
+        <v>1173671</v>
       </c>
       <c r="L14" s="11" t="n">
-        <v>1190093</v>
+        <v>1050563</v>
       </c>
       <c r="M14" s="11" t="n">
-        <v>1409309</v>
+        <v>1266827</v>
       </c>
       <c r="N14" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="11" t="n">
-        <v>1663954</v>
+        <v>1518742</v>
       </c>
       <c r="P14" s="11" t="n">
-        <v>1148372</v>
+        <v>1017310</v>
       </c>
       <c r="Q14" s="11" t="n">
         <v>509538</v>
@@ -1306,10 +1306,10 @@
         <v>46363</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>1311325</v>
+        <v>1173671</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>579428</v>
+        <v>577948</v>
       </c>
       <c r="E15" s="11" t="n">
         <v>0</v>
@@ -1330,22 +1330,22 @@
         <v>434061</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>1456693</v>
+        <v>1317558</v>
       </c>
       <c r="L15" s="11" t="n">
-        <v>1372905</v>
+        <v>1234276</v>
       </c>
       <c r="M15" s="11" t="n">
-        <v>1529811</v>
+        <v>1390443</v>
       </c>
       <c r="N15" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="11" t="n">
-        <v>1676620</v>
+        <v>1531279</v>
       </c>
       <c r="P15" s="11" t="n">
-        <v>1371054</v>
+        <v>1235347</v>
       </c>
       <c r="Q15" s="11" t="n">
         <v>509538</v>
@@ -1362,10 +1362,10 @@
         <v>46370</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>1456693</v>
+        <v>1317558</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>587443</v>
+        <v>587637</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>0</v>
@@ -1386,22 +1386,22 @@
         <v>696525</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>1347611</v>
+        <v>1208671</v>
       </c>
       <c r="L16" s="11" t="n">
-        <v>1282080</v>
+        <v>1142318</v>
       </c>
       <c r="M16" s="11" t="n">
-        <v>1409315</v>
+        <v>1270382</v>
       </c>
       <c r="N16" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="11" t="n">
-        <v>1494103</v>
+        <v>1347769</v>
       </c>
       <c r="P16" s="11" t="n">
-        <v>1343685</v>
+        <v>1208081</v>
       </c>
       <c r="Q16" s="11" t="n">
         <v>509538</v>
@@ -1418,10 +1418,10 @@
         <v>46377</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>1347611</v>
+        <v>1208671</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>566522</v>
+        <v>567175</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>0</v>
@@ -1442,22 +1442,22 @@
         <v>395578</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>1518555</v>
+        <v>1380268</v>
       </c>
       <c r="L17" s="11" t="n">
-        <v>1461156</v>
+        <v>1319636</v>
       </c>
       <c r="M17" s="11" t="n">
-        <v>1574348</v>
+        <v>1436840</v>
       </c>
       <c r="N17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="11" t="n">
-        <v>1623805</v>
+        <v>1475813</v>
       </c>
       <c r="P17" s="11" t="n">
-        <v>1588659</v>
+        <v>1455626</v>
       </c>
       <c r="Q17" s="11" t="n">
         <v>509538</v>

</xml_diff>

<commit_message>
Demo: S7 track record and data from re-exported actuals; header states case study frozen on 28 Sep for 13 weeks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXUr26jGf9sv6ye7xasg2x
</commit_message>
<xml_diff>
--- a/frontend/demo/sample/S7_sample_dataset.xlsx
+++ b/frontend/demo/sample/S7_sample_dataset.xlsx
@@ -791,7 +791,7 @@
         <v>509538</v>
       </c>
       <c r="R5" s="11" t="n">
-        <v>1388573</v>
+        <v>1498166</v>
       </c>
     </row>
     <row r="6">
@@ -847,7 +847,7 @@
         <v>509538</v>
       </c>
       <c r="R6" s="11" t="n">
-        <v>1830445</v>
+        <v>1668503</v>
       </c>
     </row>
     <row r="7">
@@ -903,7 +903,7 @@
         <v>509538</v>
       </c>
       <c r="R7" s="11" t="n">
-        <v>900266</v>
+        <v>1182312</v>
       </c>
     </row>
     <row r="8">
@@ -959,7 +959,7 @@
         <v>509538</v>
       </c>
       <c r="R8" s="11" t="n">
-        <v>1119651</v>
+        <v>1339492</v>
       </c>
     </row>
     <row r="9">
@@ -1015,7 +1015,7 @@
         <v>509538</v>
       </c>
       <c r="R9" s="11" t="n">
-        <v>1435203</v>
+        <v>1540564</v>
       </c>
     </row>
     <row r="10">
@@ -1071,7 +1071,7 @@
         <v>509538</v>
       </c>
       <c r="R10" s="11" t="n">
-        <v>1841816</v>
+        <v>1844069</v>
       </c>
     </row>
     <row r="11">
@@ -1127,7 +1127,7 @@
         <v>509538</v>
       </c>
       <c r="R11" s="11" t="n">
-        <v>1242808</v>
+        <v>1157106</v>
       </c>
     </row>
     <row r="12">
@@ -1183,7 +1183,7 @@
         <v>509538</v>
       </c>
       <c r="R12" s="11" t="n">
-        <v>1297129</v>
+        <v>1522740</v>
       </c>
     </row>
     <row r="13">
@@ -1239,7 +1239,7 @@
         <v>509538</v>
       </c>
       <c r="R13" s="11" t="n">
-        <v>1559474</v>
+        <v>1587612</v>
       </c>
     </row>
     <row r="14">
@@ -1295,7 +1295,7 @@
         <v>509538</v>
       </c>
       <c r="R14" s="11" t="n">
-        <v>1751744</v>
+        <v>1753935</v>
       </c>
     </row>
     <row r="15">
@@ -1351,7 +1351,7 @@
         <v>509538</v>
       </c>
       <c r="R15" s="11" t="n">
-        <v>1535914</v>
+        <v>1246068</v>
       </c>
     </row>
     <row r="16">
@@ -1407,7 +1407,7 @@
         <v>509538</v>
       </c>
       <c r="R16" s="11" t="n">
-        <v>1233427</v>
+        <v>1328304</v>
       </c>
     </row>
     <row r="17">
@@ -1463,7 +1463,7 @@
         <v>509538</v>
       </c>
       <c r="R17" s="11" t="n">
-        <v>1299029</v>
+        <v>1285825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>